<commit_message>
Changed features  to zig zag layout
</commit_message>
<xml_diff>
--- a/docs/Web pages.xlsx
+++ b/docs/Web pages.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\Pegboard.Web\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F23DD58-2D36-4A9F-9CC7-EE0A614773E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96F9B4B-BC48-4B2A-80DB-0B6CB46ABDCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DA042D2E-F3BD-4BD6-B120-4D79492D7016}"/>
+    <workbookView xWindow="-38510" yWindow="-9750" windowWidth="38620" windowHeight="21100" xr2:uid="{DA042D2E-F3BD-4BD6-B120-4D79492D7016}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 

</xml_diff>